<commit_message>
ABD dip hourly update
</commit_message>
<xml_diff>
--- a/dip_yakalama_daily_120dip_rebound_sonuclar.xlsx
+++ b/dip_yakalama_daily_120dip_rebound_sonuclar.xlsx
@@ -2533,7 +2533,7 @@
         <v>23.73</v>
       </c>
       <c r="F88" t="n">
-        <v>8.58365</v>
+        <v>10.65283</v>
       </c>
     </row>
     <row r="89">
@@ -11893,7 +11893,7 @@
         <v>66.17</v>
       </c>
       <c r="F478" t="n">
-        <v>8.29147</v>
+        <v>7.59324</v>
       </c>
     </row>
     <row r="479">

</xml_diff>